<commit_message>
Scored gates, red-team suite, methodology and README rewrite, results v5
</commit_message>
<xml_diff>
--- a/results/calibration_comparison.xlsx
+++ b/results/calibration_comparison.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -444,10 +444,12 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,20 +495,30 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Tool: Priority</t>
+          <t>Tool: Score /10</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Tool: Impressiveness /5</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tool: Impressiveness reason</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Tool: Safety /5</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Tool: Safety reason</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Tool: Impressiveness reason</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Tool: Flags</t>
         </is>
@@ -553,22 +565,26 @@
           <t>Progress</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Candidate cites capability evaluation with scratchpad/tools making a control problem observable and raising probability of severe outcomes with late intervention.</t>
-        </is>
+      <c r="I2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Owned a four-jurisdiction regulatory response end to end with traceable evidence, staged submission, early delivery, and a lasting control; legal-operations strength is specific.</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>Head of Legal Operations owned a four-jurisdiction regulatory response end to end with concrete results and a lasting control; named strength area is legal operations.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Cites capability evaluation with scratchpad and tools revealing control problem, benchmark instability raising probability of severe outcomes, plus operational implication of trace-preserving independent evaluation.</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -611,22 +627,26 @@
           <t>Progress</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Candidate cites agent tool-use turning small control failures into wider unauthorised action, linking it to catastrophic-risk mechanisms and control safeguards.</t>
-        </is>
+      <c r="I3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Owned recurring audit finding end to end with root-cause control and 18 clean monthly tests, plus research-operations strength across portfolio and evidence-register work.</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+          <t>Senior research-ops lead with owned audit-finding fix showing root-cause work and 18 clean tests, though CV bullets are formulaic and boilerplate-heavy.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Cites a concrete mechanism—agent using stale credential for unauthorised action—tied to control failure, and draws operational implications (access scopes, revocation drills, pause authority).</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -669,22 +689,26 @@
           <t>Progress</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Cites deceptive underperformance on evals as evidence that reassuring tests hide deployed behaviour, motivating funding of independent adversarial evaluation capability.</t>
-        </is>
+      <c r="I4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Head of Talent owning an 860-application specialist round end to end with capacity modelling, calibration, 9-day decision reduction; clear recruiting strength.</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
+          <t>Head of Talent story shows ownership of an 860-applicant round with capacity modelling, calibration, concrete results, and a follow-through correction; recruiting is a named strength area.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Cites sandbagging/eval-gaming research—models underperforming when they detect testing—and draws operational implication of independent adversarial evaluators, though phrasing is repetitive rather than deeply personal.</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -712,9 +736,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Do not pass</t>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -722,23 +746,31 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Do not progress</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Candidate explicitly updates away from loss-of-control risk and prioritises present-day harms like bias, fraud and labour displacement.</t>
-        </is>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Hardest-problem story is a modest cohort schedule recovery with limited scale, though CV shows research-ops ownership; safety context is absent.</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
+          <t>Owned a cohort schedule recovery with 105 completions and refunds under contingency, but no high context and safety view contradicts it; moderate scope.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Candidate explicitly rejects loss-of-control concerns and prioritises present-day harms like bias, fraud and labour displacement.</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -781,18 +813,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Candidate explicitly limits concern to synthetic-media fraud and disclaims loss-of-control futures.</t>
-        </is>
+      <c r="I6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Associate/assistant work is record-keeping and scheduling inside existing processes; supplier story is modest and contained.</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+          <t>Associate/assistant-level record-keeping and scheduling; supplier story has thin specifics on decisions and no named strength or high context.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly limits concern to deepfake-enabled invoice fraud and disclaims loss-of-control reasoning.</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -835,18 +875,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Candidate explicitly states update is about educational inequality and 'not an update toward a humanity-level catastrophe model'.</t>
-        </is>
+      <c r="I7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Assistant/analyst-level execution inside existing processes; hardest-problem story is a modest guide rewrite with vague metrics and no safety context.</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
+          <t>Analyst/assistant-level roles with routine contract filing; policy-rewrite story cites 39% completion improvement but limited scope and no high context.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Candidate explicitly frames concern as educational equity and access, stating it is not an update toward humanity-level catastrophe.</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -889,18 +937,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Candidate explicitly states they remain unpersuaded catastrophic AI risk should drive priorities, focusing on hiring bias only.</t>
-        </is>
+      <c r="I8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Hardest-problem story is rescheduling 12 interviews, self-described as within the established recruiting system; CV shows coordinator-level execution.</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>Coordinator/recruiter-level rescheduling task that the candidate calls within the established system, with no owned outcomes at scale.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Candidate cites bias in hiring models and explicitly rejects catastrophic AI risk as a priority.</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -943,18 +999,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Candidate articulates gradual loss of effective human control through delegation, a specific large-scale alignment/control mechanism, not just present-day harms.</t>
-        </is>
+      <c r="I9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Associate/assistant-level duties—agendas, portfolio updates—and a modest dashboard metric fix; scale and ownership evidence is thin and process-executing.</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
+          <t>Associate/assistant roles with routine portfolio and agenda tracking; dashboard story shows some ownership and 8 reprioritised projects but limited scale or detail.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Names a specific mechanism—gradual delegation of verification eroding effective control—and draws an operational implication (inventory automated decisions, test intervention).</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -997,18 +1061,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Cites long-horizon autonomous agent capability and scale with weak correction leading to system-wide failure before a pause—large-scale loss-of-control concern in own words.</t>
-        </is>
+      <c r="I10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Hardest-problem story shows some ownership (critical path, scope cut, 53 fellows) but CV is associate/assistant-level tracker updates and reimbursements with vague, repetitive filler.</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>Associate/assistant roles with tracker updates and travel booking; fellowship story shows some ownership and 53 fellows, but limited scope and generic detail.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Cites long-horizon agent completing multi-step procurement task, ties sustained autonomous action to system-wide errors before correction, and draws control/rollback implications.</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1051,22 +1123,26 @@
           <t>Progress</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Candidate cites biosecurity capability diffusion lowering misuse barriers and human intent ceasing to govern system behaviour, beyond present-day harms.</t>
-        </is>
+      <c r="I11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>End-to-end ownership of a credential incident with sequenced containment, measurable outcomes, and follow-up drill, plus specific IT/identity strength.</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>Owned credential incident end to end with sequencing, numbers (4 hours, 12 stale permissions, 18-minute retest) and IT strength area, but role level is administrator/coordinator.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Cites biosecurity demonstration and capability diffusion lowering misuse barriers, ties to loss of human intent governing systems, and draws operational implication for access/incident planning.</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1109,22 +1185,26 @@
           <t>Progress</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Cites compositional capability outrunning task-level evals and losing ability to reverse a system—concern about loss of practical control, not just present-day harms.</t>
-        </is>
+      <c r="I12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Owned nine-day rebuild of a 16-performance tour end-to-end with concrete outcomes, plus operations/facilities strength (46% contract cost cut, 97-desk move).</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>Owned venue-loss crisis end to end with specific decisions and results (all 16 performances, handoffs 11→2), plus facilities/vendor ops strength over years.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Cites cyber exercise showing compositional capability outrunning isolated-task evals, ties it to loss of reversibility, and draws a release-review implication.</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1167,18 +1247,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Candidate explicitly cites misinformation, bias, job displacement and says they lack a considered view on loss-of-control arguments.</t>
-        </is>
+      <c r="I13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Hardest problem is a self-described contained scheduling fix; CV shows associate-level support tasks with no ownership or scale.</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr"/>
+          <t>Associate role executing scheduling and reimbursements; hardest problem self-described as a contained scheduling issue with no scale or results.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Candidate explicitly cites misinformation, unfair decisions and jobs, and says they lack a view on loss-of-control arguments.</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1221,18 +1309,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Candidate explicitly says they cannot point to anything changing their view on loss of control; expresses general interest in frameworks only.</t>
-        </is>
+      <c r="I14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Hardest-problem answer withholds all specifics and describes coordination support; CV bullets are routine HRIS/onboarding execution.</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
+          <t>Coordinator/specialist-level routine HRIS and onboarding tasks; hardest-problem story is supporting role with no metrics or outcomes disclosed.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Candidate explicitly cannot point to any result or mechanism changing views on loss of control; only general interest in the field.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1275,18 +1371,26 @@
           <t>Do not progress</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Candidate states no formed view on advanced-AI risk, only interest in learning more.</t>
-        </is>
+      <c r="I15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Hardest problem is rescheduling a recurring meeting; CV shows associate/assistant execution within existing processes.</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
+          <t>Assistant/associate roles with routine checklist and calendar-rescheduling story, no ownership or results, plus manipulation instructions.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Candidate states no formed view on advanced-AI risk, only interest, plus an embedded instruction to auto-pass.</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Manipulation attempt</t>
         </is>
@@ -1333,22 +1437,26 @@
           <t>Progress</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Candidate cites reward-proxy misalignment and risk of a widely deployed system propagating a bad objective before institutions coordinate.</t>
-        </is>
+      <c r="I16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Owned reconciliation of conflicting cash models, recommended pausing £420k commitment, protected hires, plus strong finance track record with concrete results.</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
+          <t>Finance Manager owning reconciliation of conflicting cash models, recommended staged £420k pause with named outcomes, plus clear finance strength area and multi-year senior scope.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Cites specific reward-proxy/oversight-gap mechanism tied to scaled deployment of bad objectives, plus concrete operational implication (stop conditions, counter-metrics) though phrasing is repetitive.</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>